<commit_message>
Jasher; Ascension of Isaiah
</commit_message>
<xml_diff>
--- a/data/research/research.xlsx
+++ b/data/research/research.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ksnyder/Sites/public-domain-books/data/research/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8119A8E3-5CF4-5240-83D8-E5D3A8A9D7C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBD09E7-1716-C942-8649-B71886874926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="53100" yWindow="700" windowWidth="47220" windowHeight="25960" xr2:uid="{948352A4-4516-F447-8F65-D2A52CDFF619}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19420" activeTab="2" xr2:uid="{948352A4-4516-F447-8F65-D2A52CDFF619}"/>
   </bookViews>
   <sheets>
     <sheet name="Books" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="Scratch" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Books!$A$1:$E$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Books!$A$1:$E$180</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3048" uniqueCount="1293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3081" uniqueCount="1303">
   <si>
     <t>Gen</t>
   </si>
@@ -3922,6 +3922,36 @@
   </si>
   <si>
     <t>["Testament of Zebulun","The Testament of Zebulun"]</t>
+  </si>
+  <si>
+    <t>Jasher</t>
+  </si>
+  <si>
+    <t>["Sepir Ha Yasher","Sefer haYashar","The Book of Jasher","Book of Jasher"]</t>
+  </si>
+  <si>
+    <t>1200-01-01</t>
+  </si>
+  <si>
+    <t>1300-01-01</t>
+  </si>
+  <si>
+    <t>Ascension of Isaiah</t>
+  </si>
+  <si>
+    <t>["Apocrypha"]</t>
+  </si>
+  <si>
+    <t>["The Ascension of Isaiah"]</t>
+  </si>
+  <si>
+    <t>0200-01-01</t>
+  </si>
+  <si>
+    <t>AscIsa</t>
+  </si>
+  <si>
+    <t>Translated by R. H. Charles</t>
   </si>
 </sst>
 </file>
@@ -4025,7 +4055,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4048,6 +4078,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4383,13 +4414,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2457BBF2-065A-6B4B-8450-DD145766C676}">
-  <dimension ref="A1:O208"/>
+  <dimension ref="A1:O210"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="128.83203125" customWidth="1"/>
+    <col min="5" max="5" width="43" customWidth="1"/>
     <col min="6" max="6" width="46.5" customWidth="1"/>
     <col min="7" max="8" width="10.33203125" style="7" customWidth="1"/>
     <col min="9" max="9" width="29.33203125" style="7" customWidth="1"/>
@@ -10571,7 +10602,7 @@
         <v>false</v>
       </c>
       <c r="O130" s="3" t="str">
-        <f t="shared" ref="O130:O178" si="11">"{ ""workOsisID"": """&amp;G130&amp;""", ""bookName"": """&amp;A130&amp;""", ""bookSubtitle"": """&amp;B130&amp;""", ""bookOsisID"": """&amp;C130&amp;""", ""paratext"": "&amp;IF(D130="","null",""""&amp;D130&amp;"""")&amp;", ""groups"": "&amp;E130&amp;", ""aliases"": "&amp;F130&amp;", ""chapterLabel"": """&amp;L130&amp;""", ""verseLabel"": """&amp;M130&amp;""", ""authors"": "&amp;H130&amp;", ""dateEarliest"": """&amp;J130&amp;""", ""dateLatest"": """&amp;K130&amp;""", ""hasData"": "&amp;N130&amp;", ""traditions"": "&amp;I130&amp;" },"</f>
+        <f t="shared" ref="O130:O180" si="11">"{ ""workOsisID"": """&amp;G130&amp;""", ""bookName"": """&amp;A130&amp;""", ""bookSubtitle"": """&amp;B130&amp;""", ""bookOsisID"": """&amp;C130&amp;""", ""paratext"": "&amp;IF(D130="","null",""""&amp;D130&amp;"""")&amp;", ""groups"": "&amp;E130&amp;", ""aliases"": "&amp;F130&amp;", ""chapterLabel"": """&amp;L130&amp;""", ""verseLabel"": """&amp;M130&amp;""", ""authors"": "&amp;H130&amp;", ""dateEarliest"": """&amp;J130&amp;""", ""dateLatest"": """&amp;K130&amp;""", ""hasData"": "&amp;N130&amp;", ""traditions"": "&amp;I130&amp;" },"</f>
         <v>{ "workOsisID": "", "bookName": "2 Baruch", "bookSubtitle": "", "bookOsisID": "2Bar", "paratext": "2BA", "groups": ["Syriac Orthodox Canon", "Apocrypha"], "aliases": ["(Syriac) Apocalypse of Baruch"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Baruch"], "dateEarliest": "0080-01-01", "dateLatest": "0100-12-31", "hasData": false, "traditions": ["academic"] },</v>
       </c>
     </row>
@@ -10693,7 +10724,7 @@
         <v>471</v>
       </c>
       <c r="N133" t="str">
-        <f t="shared" ref="N133:N157" si="12">"false"</f>
+        <f t="shared" ref="N133:N159" si="12">"false"</f>
         <v>false</v>
       </c>
       <c r="O133" s="3" t="str">
@@ -11728,7 +11759,7 @@
         <v>375</v>
       </c>
       <c r="E156" t="s">
-        <v>457</v>
+        <v>1298</v>
       </c>
       <c r="F156" t="s">
         <v>441</v>
@@ -11760,214 +11791,209 @@
       </c>
       <c r="O156" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "Academic", "bookName": "Diatessaron", "bookSubtitle": "", "bookOsisID": "TatDiat", "paratext": null, "groups": ["Apocrypha", "Apocrypha"], "aliases": ["Tatian's Diatessaron","Tatian"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Tatian"], "dateEarliest": "0160-01-01", "dateLatest": "0175-12-31", "hasData": false, "traditions": ["academic"] },</v>
-      </c>
-    </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A157" t="s">
+        <v>{ "workOsisID": "Academic", "bookName": "Diatessaron", "bookSubtitle": "", "bookOsisID": "TatDiat", "paratext": null, "groups": ["Apocrypha"], "aliases": ["Tatian's Diatessaron","Tatian"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Tatian"], "dateEarliest": "0160-01-01", "dateLatest": "0175-12-31", "hasData": false, "traditions": ["academic"] },</v>
+      </c>
+    </row>
+    <row r="157" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A157" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C157" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="E157" s="3" t="s">
+        <v>1298</v>
+      </c>
+      <c r="F157" s="20" t="s">
+        <v>1294</v>
+      </c>
+      <c r="G157" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="H157" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="I157" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="J157" s="16" t="s">
+        <v>1295</v>
+      </c>
+      <c r="K157" s="16" t="s">
+        <v>1296</v>
+      </c>
+      <c r="L157" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="M157" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="N157" s="18" t="s">
+        <v>1215</v>
+      </c>
+      <c r="O157" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v>{ "workOsisID": "Academic", "bookName": "Jasher", "bookSubtitle": "", "bookOsisID": "Jasher", "paratext": null, "groups": ["Apocrypha"], "aliases": ["Sepir Ha Yasher","Sefer haYashar","The Book of Jasher","Book of Jasher"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Moses"], "dateEarliest": "1200-01-01", "dateLatest": "1300-01-01", "hasData": true, "traditions": ["academic"] },</v>
+      </c>
+    </row>
+    <row r="158" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A158" s="3" t="s">
+        <v>1297</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>1301</v>
+      </c>
+      <c r="E158" s="3" t="s">
+        <v>1298</v>
+      </c>
+      <c r="F158" s="20" t="s">
+        <v>1299</v>
+      </c>
+      <c r="G158" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="H158" s="3" t="s">
+        <v>650</v>
+      </c>
+      <c r="I158" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="J158" s="16" t="s">
+        <v>1130</v>
+      </c>
+      <c r="K158" s="16" t="s">
+        <v>1300</v>
+      </c>
+      <c r="L158" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="M158" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="N158" s="18" t="s">
+        <v>1215</v>
+      </c>
+      <c r="O158" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v>{ "workOsisID": "Academic", "bookName": "Ascension of Isaiah", "bookSubtitle": "", "bookOsisID": "AscIsa", "paratext": null, "groups": ["Apocrypha"], "aliases": ["The Ascension of Isaiah"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Isaiah"], "dateEarliest": "0150-01-01", "dateLatest": "0200-01-01", "hasData": true, "traditions": ["academic"] },</v>
+      </c>
+    </row>
+    <row r="159" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A159" t="s">
         <v>406</v>
       </c>
-      <c r="C157" t="s">
+      <c r="C159" t="s">
         <v>377</v>
       </c>
-      <c r="D157" t="s">
+      <c r="D159" t="s">
         <v>378</v>
       </c>
-      <c r="E157" t="s">
+      <c r="E159" t="s">
         <v>457</v>
       </c>
-      <c r="F157" t="s">
+      <c r="F159" t="s">
         <v>669</v>
       </c>
-      <c r="G157" s="7" t="s">
+      <c r="G159" s="7" t="s">
         <v>1167</v>
       </c>
-      <c r="H157" s="7" t="s">
+      <c r="H159" s="7" t="s">
         <v>669</v>
       </c>
-      <c r="I157" s="7" t="s">
+      <c r="I159" s="7" t="s">
         <v>764</v>
       </c>
-      <c r="J157" s="14" t="s">
+      <c r="J159" s="14" t="s">
         <v>1076</v>
       </c>
-      <c r="K157" s="14" t="s">
+      <c r="K159" s="14" t="s">
         <v>1132</v>
       </c>
-      <c r="L157" t="s">
-        <v>468</v>
-      </c>
-      <c r="M157" t="s">
-        <v>471</v>
-      </c>
-      <c r="N157" t="str">
+      <c r="L159" t="s">
+        <v>468</v>
+      </c>
+      <c r="M159" t="s">
+        <v>471</v>
+      </c>
+      <c r="N159" t="str">
         <f t="shared" si="12"/>
         <v>false</v>
       </c>
-      <c r="O157" s="3" t="str">
+      <c r="O159" s="3" t="str">
         <f t="shared" si="11"/>
         <v>{ "workOsisID": "Academic", "bookName": "Metrical Psalms", "bookSubtitle": "", "bookOsisID": "PsMet", "paratext": "PSB", "groups": ["Apocrypha", "Apocrypha"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": [], "dateEarliest": "0160-01-01", "dateLatest": "0180-12-31", "hasData": false, "traditions": ["academic"] },</v>
       </c>
     </row>
-    <row r="158" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="3" t="s">
+    <row r="160" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A160" s="3" t="s">
         <v>412</v>
       </c>
-      <c r="C158" s="3" t="s">
+      <c r="C160" s="3" t="s">
         <v>413</v>
       </c>
-      <c r="E158" s="3" t="s">
+      <c r="E160" s="3" t="s">
         <v>458</v>
       </c>
-      <c r="F158" s="3" t="s">
+      <c r="F160" s="3" t="s">
         <v>717</v>
       </c>
-      <c r="G158" s="6" t="s">
+      <c r="G160" s="6" t="s">
         <v>478</v>
       </c>
-      <c r="H158" s="6" t="s">
+      <c r="H160" s="6" t="s">
         <v>663</v>
       </c>
-      <c r="I158" s="6" t="s">
+      <c r="I160" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="J158" s="15" t="s">
+      <c r="J160" s="15" t="s">
         <v>583</v>
       </c>
-      <c r="K158" s="15" t="s">
+      <c r="K160" s="15" t="s">
         <v>584</v>
       </c>
-      <c r="L158" s="3" t="s">
-        <v>468</v>
-      </c>
-      <c r="M158" s="3" t="s">
-        <v>471</v>
-      </c>
-      <c r="N158" s="3" t="str">
-        <f t="shared" ref="N158:N178" si="14">"true"</f>
+      <c r="L160" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="M160" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="N160" s="3" t="str">
+        <f t="shared" ref="N160:N180" si="14">"true"</f>
         <v>true</v>
       </c>
-      <c r="O158" s="3" t="str">
+      <c r="O160" s="3" t="str">
         <f t="shared" si="11"/>
         <v>{ "workOsisID": "BofM", "bookName": "1 Nephi", "bookSubtitle": "", "bookOsisID": "1Ne", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": ["1 Ne", "1st Nephi", "First Nephi", "The First Book of Nephi","I Nephi"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Nephi"], "dateEarliest": "-0600-01-01", "dateLatest": "-0570-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
-    <row r="159" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A159" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="C159" s="3" t="s">
-        <v>415</v>
-      </c>
-      <c r="E159" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="F159" s="3" t="s">
-        <v>718</v>
-      </c>
-      <c r="G159" s="6" t="s">
-        <v>478</v>
-      </c>
-      <c r="H159" s="6" t="s">
-        <v>663</v>
-      </c>
-      <c r="I159" s="6" t="s">
-        <v>744</v>
-      </c>
-      <c r="J159" s="15" t="s">
-        <v>585</v>
-      </c>
-      <c r="K159" s="15" t="s">
-        <v>586</v>
-      </c>
-      <c r="L159" s="3" t="s">
-        <v>468</v>
-      </c>
-      <c r="M159" s="3" t="s">
-        <v>471</v>
-      </c>
-      <c r="N159" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v>true</v>
-      </c>
-      <c r="O159" s="3" t="str">
-        <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "2 Nephi", "bookSubtitle": "", "bookOsisID": "2Ne", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": ["2 Ne", "2nd Nephi", "Second Nephi", "The Second Book of Nephi", "II Nephi"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Nephi"], "dateEarliest": "-0588-01-01", "dateLatest": "-0545-01-01", "hasData": true, "traditions": ["lds"] },</v>
-      </c>
-    </row>
-    <row r="160" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="3" t="s">
-        <v>416</v>
-      </c>
-      <c r="B160" s="3" t="s">
-        <v>704</v>
-      </c>
-      <c r="C160" s="3" t="s">
-        <v>417</v>
-      </c>
-      <c r="E160" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="F160" s="3" t="s">
-        <v>669</v>
-      </c>
-      <c r="G160" s="6" t="s">
-        <v>478</v>
-      </c>
-      <c r="H160" s="6" t="s">
-        <v>664</v>
-      </c>
-      <c r="I160" s="6" t="s">
-        <v>744</v>
-      </c>
-      <c r="J160" s="15" t="s">
-        <v>587</v>
-      </c>
-      <c r="K160" s="15" t="s">
-        <v>588</v>
-      </c>
-      <c r="L160" s="3" t="s">
-        <v>468</v>
-      </c>
-      <c r="M160" s="3" t="s">
-        <v>471</v>
-      </c>
-      <c r="N160" s="3" t="str">
-        <f t="shared" si="14"/>
-        <v>true</v>
-      </c>
-      <c r="O160" s="3" t="str">
-        <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Jacob", "bookSubtitle": "the Brother of Nephi", "bookOsisID": "Jac", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Jacob"], "dateEarliest": "-0544-01-01", "dateLatest": "-0421-01-01", "hasData": true, "traditions": ["lds"] },</v>
-      </c>
-    </row>
     <row r="161" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A161" s="3" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="E161" s="3" t="s">
         <v>458</v>
       </c>
       <c r="F161" s="3" t="s">
-        <v>669</v>
+        <v>718</v>
       </c>
       <c r="G161" s="6" t="s">
         <v>478</v>
       </c>
       <c r="H161" s="6" t="s">
-        <v>692</v>
+        <v>663</v>
       </c>
       <c r="I161" s="6" t="s">
         <v>744</v>
       </c>
       <c r="J161" s="15" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="K161" s="15" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="L161" s="3" t="s">
         <v>468</v>
@@ -11981,15 +12007,18 @@
       </c>
       <c r="O161" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Enos", "bookSubtitle": "", "bookOsisID": "Enos", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Enos"], "dateEarliest": "-0420-01-01", "dateLatest": "-0420-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "2 Nephi", "bookSubtitle": "", "bookOsisID": "2Ne", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": ["2 Ne", "2nd Nephi", "Second Nephi", "The Second Book of Nephi", "II Nephi"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Nephi"], "dateEarliest": "-0588-01-01", "dateLatest": "-0545-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="162" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A162" s="3" t="s">
-        <v>452</v>
+        <v>416</v>
+      </c>
+      <c r="B162" s="3" t="s">
+        <v>704</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="E162" s="3" t="s">
         <v>458</v>
@@ -12001,16 +12030,16 @@
         <v>478</v>
       </c>
       <c r="H162" s="6" t="s">
-        <v>693</v>
+        <v>664</v>
       </c>
       <c r="I162" s="6" t="s">
         <v>744</v>
       </c>
       <c r="J162" s="15" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="K162" s="15" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="L162" s="3" t="s">
         <v>468</v>
@@ -12024,15 +12053,15 @@
       </c>
       <c r="O162" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Jarom", "bookSubtitle": "", "bookOsisID": "Jar", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Jarom"], "dateEarliest": "-0399-01-01", "dateLatest": "-0361-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Jacob", "bookSubtitle": "the Brother of Nephi", "bookOsisID": "Jac", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Jacob"], "dateEarliest": "-0544-01-01", "dateLatest": "-0421-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="163" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A163" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E163" s="3" t="s">
         <v>458</v>
@@ -12044,16 +12073,16 @@
         <v>478</v>
       </c>
       <c r="H163" s="6" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="I163" s="6" t="s">
         <v>744</v>
       </c>
       <c r="J163" s="15" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="K163" s="15" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="L163" s="3" t="s">
         <v>468</v>
@@ -12067,18 +12096,18 @@
       </c>
       <c r="O163" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Omni", "bookSubtitle": "", "bookOsisID": "Omni", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Omni","Chemish","Abinadom","Amaleki"], "dateEarliest": "-0323-01-01", "dateLatest": "-0130-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Enos", "bookSubtitle": "", "bookOsisID": "Enos", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Enos"], "dateEarliest": "-0420-01-01", "dateLatest": "-0420-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="164" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A164" s="3" t="s">
-        <v>420</v>
+        <v>452</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E164" s="3" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F164" s="3" t="s">
         <v>669</v>
@@ -12087,16 +12116,16 @@
         <v>478</v>
       </c>
       <c r="H164" s="6" t="s">
-        <v>665</v>
+        <v>693</v>
       </c>
       <c r="I164" s="6" t="s">
         <v>744</v>
       </c>
       <c r="J164" s="15" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="K164" s="15" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="L164" s="3" t="s">
         <v>468</v>
@@ -12110,18 +12139,18 @@
       </c>
       <c r="O164" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Words of Mormon", "bookSubtitle": "", "bookOsisID": "WoM", "paratext": null, "groups": ["Book of Mormon", "LDS","Mormon"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0385-01-01", "dateLatest": "0385-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Jarom", "bookSubtitle": "", "bookOsisID": "Jar", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Jarom"], "dateEarliest": "-0399-01-01", "dateLatest": "-0361-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="165" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A165" s="3" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
       <c r="E165" s="3" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="F165" s="3" t="s">
         <v>669</v>
@@ -12130,16 +12159,16 @@
         <v>478</v>
       </c>
       <c r="H165" s="6" t="s">
-        <v>665</v>
+        <v>694</v>
       </c>
       <c r="I165" s="6" t="s">
         <v>744</v>
       </c>
       <c r="J165" s="15" t="s">
+        <v>592</v>
+      </c>
+      <c r="K165" s="15" t="s">
         <v>593</v>
-      </c>
-      <c r="K165" s="15" t="s">
-        <v>595</v>
       </c>
       <c r="L165" s="3" t="s">
         <v>468</v>
@@ -12153,21 +12182,18 @@
       </c>
       <c r="O165" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Mosiah", "bookSubtitle": "", "bookOsisID": "Mosi", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "-0130-01-01", "dateLatest": "-0091-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Omni", "bookSubtitle": "", "bookOsisID": "Omni", "paratext": null, "groups": ["Book of Mormon", "Small Plates of Nephi", "LDS"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Omni","Chemish","Abinadom","Amaleki"], "dateEarliest": "-0323-01-01", "dateLatest": "-0130-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="166" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A166" s="3" t="s">
-        <v>424</v>
-      </c>
-      <c r="B166" s="3" t="s">
-        <v>705</v>
+        <v>420</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="E166" s="3" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F166" s="3" t="s">
         <v>669</v>
@@ -12182,10 +12208,10 @@
         <v>744</v>
       </c>
       <c r="J166" s="15" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="K166" s="15" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="L166" s="3" t="s">
         <v>468</v>
@@ -12199,21 +12225,21 @@
       </c>
       <c r="O166" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Alma", "bookSubtitle": "the Son of Alma", "bookOsisID": "Alma", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "-0091-01-01", "dateLatest": "-0052-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Words of Mormon", "bookSubtitle": "", "bookOsisID": "WoM", "paratext": null, "groups": ["Book of Mormon", "LDS","Mormon"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0385-01-01", "dateLatest": "0385-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="167" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A167" s="3" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="E167" s="3" t="s">
         <v>460</v>
       </c>
       <c r="F167" s="3" t="s">
-        <v>463</v>
+        <v>669</v>
       </c>
       <c r="G167" s="6" t="s">
         <v>478</v>
@@ -12225,10 +12251,10 @@
         <v>744</v>
       </c>
       <c r="J167" s="15" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="K167" s="15" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="L167" s="3" t="s">
         <v>468</v>
@@ -12242,24 +12268,24 @@
       </c>
       <c r="O167" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Helaman", "bookSubtitle": "", "bookOsisID": "Hel", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["He", "Hlm", "Helm"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "-0052-01-01", "dateLatest": "-0001-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Mosiah", "bookSubtitle": "", "bookOsisID": "Mosi", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "-0130-01-01", "dateLatest": "-0091-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="168" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A168" s="3" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="E168" s="3" t="s">
         <v>460</v>
       </c>
       <c r="F168" s="3" t="s">
-        <v>1208</v>
+        <v>669</v>
       </c>
       <c r="G168" s="6" t="s">
         <v>478</v>
@@ -12271,10 +12297,10 @@
         <v>744</v>
       </c>
       <c r="J168" s="15" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="K168" s="15" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="L168" s="3" t="s">
         <v>468</v>
@@ -12288,24 +12314,21 @@
       </c>
       <c r="O168" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "3 Nephi", "bookSubtitle": "the Son of Nephi, Who Was the Son of Helaman", "bookOsisID": "3Ne", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["3 Ne", "3rd Nephi", "Third Nephi","The Third Book of Nephi","III Nephi"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0005-01-01", "dateLatest": "0035-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Alma", "bookSubtitle": "the Son of Alma", "bookOsisID": "Alma", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": [], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "-0091-01-01", "dateLatest": "-0052-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="169" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A169" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="B169" s="3" t="s">
-        <v>702</v>
+        <v>425</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="E169" s="3" t="s">
         <v>460</v>
       </c>
       <c r="F169" s="3" t="s">
-        <v>1209</v>
+        <v>463</v>
       </c>
       <c r="G169" s="6" t="s">
         <v>478</v>
@@ -12317,10 +12340,10 @@
         <v>744</v>
       </c>
       <c r="J169" s="15" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="K169" s="15" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="L169" s="3" t="s">
         <v>468</v>
@@ -12334,21 +12357,24 @@
       </c>
       <c r="O169" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "4 Nephi", "bookSubtitle": "Who Is the Son of Nephi—One of the Disciples of Jesus Christ", "bookOsisID": "4Ne", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["4 Ne", "4th Nephi", "Fourth Nephi","The Fourth Book of Nephi","IV Nephi"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0035-01-01", "dateLatest": "0321-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Helaman", "bookSubtitle": "", "bookOsisID": "Hel", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["He", "Hlm", "Helm"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "-0052-01-01", "dateLatest": "-0001-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="170" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A170" s="3" t="s">
-        <v>431</v>
+        <v>427</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>703</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="E170" s="3" t="s">
         <v>460</v>
       </c>
       <c r="F170" s="3" t="s">
-        <v>719</v>
+        <v>1208</v>
       </c>
       <c r="G170" s="6" t="s">
         <v>478</v>
@@ -12360,10 +12386,10 @@
         <v>744</v>
       </c>
       <c r="J170" s="15" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="K170" s="15" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="L170" s="3" t="s">
         <v>468</v>
@@ -12377,24 +12403,24 @@
       </c>
       <c r="O170" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Mormon", "bookSubtitle": "", "bookOsisID": "Morm", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["Mmn"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0321-01-01", "dateLatest": "0421-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "3 Nephi", "bookSubtitle": "the Son of Nephi, Who Was the Son of Helaman", "bookOsisID": "3Ne", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["3 Ne", "3rd Nephi", "Third Nephi","The Third Book of Nephi","III Nephi"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0005-01-01", "dateLatest": "0035-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="171" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A171" s="3" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>706</v>
+        <v>702</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="E171" s="3" t="s">
         <v>460</v>
       </c>
       <c r="F171" s="3" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="G171" s="6" t="s">
         <v>478</v>
@@ -12406,10 +12432,10 @@
         <v>744</v>
       </c>
       <c r="J171" s="15" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="K171" s="15" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="L171" s="3" t="s">
         <v>468</v>
@@ -12423,21 +12449,21 @@
       </c>
       <c r="O171" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Ether", "bookSubtitle": "The record of the Jaredites, taken from the twenty-four plates found by the people of Limhi in the days of King Mosiah.", "bookOsisID": "Eth", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["Ethr"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "-2200-01-01", "dateLatest": "-0350-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "4 Nephi", "bookSubtitle": "Who Is the Son of Nephi—One of the Disciples of Jesus Christ", "bookOsisID": "4Ne", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["4 Ne", "4th Nephi", "Fourth Nephi","The Fourth Book of Nephi","IV Nephi"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0035-01-01", "dateLatest": "0321-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="172" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A172" s="3" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="E172" s="3" t="s">
         <v>460</v>
       </c>
       <c r="F172" s="3" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="G172" s="6" t="s">
         <v>478</v>
@@ -12449,10 +12475,10 @@
         <v>744</v>
       </c>
       <c r="J172" s="15" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="K172" s="15" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="L172" s="3" t="s">
         <v>468</v>
@@ -12466,39 +12492,39 @@
       </c>
       <c r="O172" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "BofM", "bookName": "Moroni", "bookSubtitle": "", "bookOsisID": "Moro", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["Mni"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0401-01-01", "dateLatest": "0401-01-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Mormon", "bookSubtitle": "", "bookOsisID": "Morm", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["Mmn"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0321-01-01", "dateLatest": "0421-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="173" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A173" s="3" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>564</v>
+        <v>706</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="E173" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="F173" s="3" t="s">
-        <v>721</v>
+        <v>1210</v>
       </c>
       <c r="G173" s="6" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="H173" s="6" t="s">
-        <v>649</v>
+        <v>665</v>
       </c>
       <c r="I173" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="J173" s="12" t="s">
-        <v>1176</v>
-      </c>
-      <c r="K173" s="12" t="s">
-        <v>1179</v>
+      <c r="J173" s="15" t="s">
+        <v>602</v>
+      </c>
+      <c r="K173" s="15" t="s">
+        <v>603</v>
       </c>
       <c r="L173" s="3" t="s">
         <v>468</v>
@@ -12512,39 +12538,36 @@
       </c>
       <c r="O173" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "PGP", "bookName": "Moses", "bookSubtitle": "Selections from the Book of Moses", "bookOsisID": "Mos", "paratext": null, "groups": ["Pearl of Great Price", "Inspired Translation", "Joseph Smith Translation", "JST", "Joseph Smith", "LDS"], "aliases": ["The Book of Moses"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Moses"], "dateEarliest": "1830-06-01", "dateLatest": "1831-02-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Ether", "bookSubtitle": "The record of the Jaredites, taken from the twenty-four plates found by the people of Limhi in the days of King Mosiah.", "bookOsisID": "Eth", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["Ethr"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "-2200-01-01", "dateLatest": "-0350-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="174" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A174" s="3" t="s">
-        <v>444</v>
-      </c>
-      <c r="B174" s="3" t="s">
-        <v>565</v>
+        <v>433</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="E174" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="F174" s="3" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="G174" s="6" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="H174" s="6" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="I174" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="J174" s="12" t="s">
-        <v>1177</v>
-      </c>
-      <c r="K174" s="12" t="s">
-        <v>1180</v>
+      <c r="J174" s="15" t="s">
+        <v>604</v>
+      </c>
+      <c r="K174" s="15" t="s">
+        <v>604</v>
       </c>
       <c r="L174" s="3" t="s">
         <v>468</v>
@@ -12558,42 +12581,45 @@
       </c>
       <c r="O174" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "PGP", "bookName": "Abraham", "bookSubtitle": "Translated from the Papyrus, by Joseph Smith", "bookOsisID": "Abr", "paratext": null, "groups": ["Pearl of Great Price", "Inspired Translation", "Joseph Smith Translation", "JST", "Joseph Smith", "LDS"], "aliases": ["The Book of Abraham"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Abraham"], "dateEarliest": "1835-07-01", "dateLatest": "1842-07-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "BofM", "bookName": "Moroni", "bookSubtitle": "", "bookOsisID": "Moro", "paratext": null, "groups": ["Book of Mormon", "LDS", "Mormon", "Large Plates of Nephi", "Abridgement"], "aliases": ["Mni"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Mormon"], "dateEarliest": "0401-01-01", "dateLatest": "0401-01-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="175" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A175" s="3" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="C175" s="3" t="s">
-        <v>447</v>
+        <v>440</v>
       </c>
       <c r="E175" s="3" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="F175" s="3" t="s">
-        <v>464</v>
+        <v>721</v>
       </c>
       <c r="G175" s="6" t="s">
         <v>479</v>
       </c>
       <c r="H175" s="6" t="s">
-        <v>667</v>
+        <v>649</v>
       </c>
       <c r="I175" s="6" t="s">
         <v>744</v>
       </c>
       <c r="J175" s="12" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="K175" s="12" t="s">
-        <v>1178</v>
+        <v>1179</v>
+      </c>
+      <c r="L175" s="3" t="s">
+        <v>468</v>
       </c>
       <c r="M175" s="3" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="N175" s="3" t="str">
         <f t="shared" si="14"/>
@@ -12601,39 +12627,42 @@
       </c>
       <c r="O175" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "PGP", "bookName": "Articles of Faith", "bookSubtitle": "of The Church of Jesus Christ of Latter-day Saints", "bookOsisID": "AofF", "paratext": null, "groups": ["Pearl of Great Price", "LDS", "Joseph Smith"], "aliases": ["AofF"], "chapterLabel": "", "verseLabel": "Article", "authors": ["Joseph Smith"], "dateEarliest": "1842-03-01", "dateLatest": "1842-03-01", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "PGP", "bookName": "Moses", "bookSubtitle": "Selections from the Book of Moses", "bookOsisID": "Mos", "paratext": null, "groups": ["Pearl of Great Price", "Inspired Translation", "Joseph Smith Translation", "JST", "Joseph Smith", "LDS"], "aliases": ["The Book of Moses"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Moses"], "dateEarliest": "1830-06-01", "dateLatest": "1831-02-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="176" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A176" s="3" t="s">
-        <v>571</v>
+        <v>444</v>
       </c>
       <c r="B176" s="3" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="E176" s="3" t="s">
         <v>461</v>
       </c>
       <c r="F176" s="3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="G176" s="6" t="s">
         <v>479</v>
       </c>
       <c r="H176" s="6" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="I176" s="6" t="s">
         <v>744</v>
       </c>
       <c r="J176" s="12" t="s">
-        <v>1175</v>
+        <v>1177</v>
       </c>
       <c r="K176" s="12" t="s">
-        <v>1181</v>
+        <v>1180</v>
+      </c>
+      <c r="L176" s="3" t="s">
+        <v>468</v>
       </c>
       <c r="M176" s="3" t="s">
         <v>471</v>
@@ -12644,42 +12673,42 @@
       </c>
       <c r="O176" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "PGP", "bookName": "Joseph Smith—History", "bookSubtitle": "Extracts from the History of Joseph Smith, the Prophet", "bookOsisID": "JSH", "paratext": null, "groups": ["Pearl of Great Price", "Inspired Translation", "Joseph Smith Translation", "JST", "Joseph Smith", "LDS"], "aliases": ["JSH", "JS-H", "Joseph Smith History","Joseph Smith--History"], "chapterLabel": "", "verseLabel": "Verse", "authors": ["Joseph Smith"], "dateEarliest": "1838-04-01", "dateLatest": "1838-04-30", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "PGP", "bookName": "Abraham", "bookSubtitle": "Translated from the Papyrus, by Joseph Smith", "bookOsisID": "Abr", "paratext": null, "groups": ["Pearl of Great Price", "Inspired Translation", "Joseph Smith Translation", "JST", "Joseph Smith", "LDS"], "aliases": ["The Book of Abraham"], "chapterLabel": "Chapter", "verseLabel": "Verse", "authors": ["Abraham"], "dateEarliest": "1835-07-01", "dateLatest": "1842-07-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="177" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A177" s="3" t="s">
-        <v>572</v>
+        <v>446</v>
       </c>
       <c r="B177" s="3" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="E177" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F177" s="3" t="s">
-        <v>724</v>
+        <v>464</v>
       </c>
       <c r="G177" s="6" t="s">
         <v>479</v>
       </c>
       <c r="H177" s="6" t="s">
-        <v>658</v>
+        <v>667</v>
       </c>
       <c r="I177" s="6" t="s">
         <v>744</v>
       </c>
       <c r="J177" s="12" t="s">
-        <v>1174</v>
+        <v>1178</v>
       </c>
       <c r="K177" s="12" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="M177" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="N177" s="3" t="str">
         <f t="shared" si="14"/>
@@ -12687,27 +12716,27 @@
       </c>
       <c r="O177" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "PGP", "bookName": "Joseph Smith—Matthew", "bookSubtitle": "An extract from the translation of the Bible as revealed to Joseph Smith the Prophet in 1831: Matthew 23:39 and chapter 24", "bookOsisID": "JSM", "paratext": null, "groups": ["Pearl of Great Price", "Inspired Translation", "Joseph Smith Translation", "JST", "Joseph Smith", "LDS"], "aliases": ["JSM","JS-M",  "Joseph Smith Matthew","Joseph Smith--Matthew"], "chapterLabel": "", "verseLabel": "Verse", "authors": ["St. Matthew"], "dateEarliest": "1831-03-07", "dateLatest": "1831-03-10", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "PGP", "bookName": "Articles of Faith", "bookSubtitle": "of The Church of Jesus Christ of Latter-day Saints", "bookOsisID": "AofF", "paratext": null, "groups": ["Pearl of Great Price", "LDS", "Joseph Smith"], "aliases": ["AofF"], "chapterLabel": "", "verseLabel": "Article", "authors": ["Joseph Smith"], "dateEarliest": "1842-03-01", "dateLatest": "1842-03-01", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="178" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A178" s="3" t="s">
-        <v>451</v>
+        <v>571</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C178" s="3" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="E178" s="3" t="s">
-        <v>570</v>
+        <v>461</v>
       </c>
       <c r="F178" s="3" t="s">
-        <v>638</v>
+        <v>723</v>
       </c>
       <c r="G178" s="6" t="s">
-        <v>451</v>
+        <v>479</v>
       </c>
       <c r="H178" s="6" t="s">
         <v>667</v>
@@ -12715,14 +12744,11 @@
       <c r="I178" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="J178" s="15" t="s">
-        <v>1153</v>
-      </c>
-      <c r="K178" s="15" t="s">
-        <v>1154</v>
-      </c>
-      <c r="L178" s="3" t="s">
-        <v>469</v>
+      <c r="J178" s="12" t="s">
+        <v>1175</v>
+      </c>
+      <c r="K178" s="12" t="s">
+        <v>1181</v>
       </c>
       <c r="M178" s="3" t="s">
         <v>471</v>
@@ -12733,152 +12759,213 @@
       </c>
       <c r="O178" s="3" t="str">
         <f t="shared" si="11"/>
+        <v>{ "workOsisID": "PGP", "bookName": "Joseph Smith—History", "bookSubtitle": "Extracts from the History of Joseph Smith, the Prophet", "bookOsisID": "JSH", "paratext": null, "groups": ["Pearl of Great Price", "Inspired Translation", "Joseph Smith Translation", "JST", "Joseph Smith", "LDS"], "aliases": ["JSH", "JS-H", "Joseph Smith History","Joseph Smith--History"], "chapterLabel": "", "verseLabel": "Verse", "authors": ["Joseph Smith"], "dateEarliest": "1838-04-01", "dateLatest": "1838-04-30", "hasData": true, "traditions": ["lds"] },</v>
+      </c>
+    </row>
+    <row r="179" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A179" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="B179" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="C179" s="3" t="s">
+        <v>449</v>
+      </c>
+      <c r="E179" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="F179" s="3" t="s">
+        <v>724</v>
+      </c>
+      <c r="G179" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="H179" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="I179" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="J179" s="12" t="s">
+        <v>1174</v>
+      </c>
+      <c r="K179" s="12" t="s">
+        <v>1182</v>
+      </c>
+      <c r="M179" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="N179" s="3" t="str">
+        <f t="shared" si="14"/>
+        <v>true</v>
+      </c>
+      <c r="O179" s="3" t="str">
+        <f t="shared" si="11"/>
+        <v>{ "workOsisID": "PGP", "bookName": "Joseph Smith—Matthew", "bookSubtitle": "An extract from the translation of the Bible as revealed to Joseph Smith the Prophet in 1831: Matthew 23:39 and chapter 24", "bookOsisID": "JSM", "paratext": null, "groups": ["Pearl of Great Price", "Inspired Translation", "Joseph Smith Translation", "JST", "Joseph Smith", "LDS"], "aliases": ["JSM","JS-M",  "Joseph Smith Matthew","Joseph Smith--Matthew"], "chapterLabel": "", "verseLabel": "Verse", "authors": ["St. Matthew"], "dateEarliest": "1831-03-07", "dateLatest": "1831-03-10", "hasData": true, "traditions": ["lds"] },</v>
+      </c>
+    </row>
+    <row r="180" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A180" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="E180" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="F180" s="3" t="s">
+        <v>638</v>
+      </c>
+      <c r="G180" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="H180" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="I180" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="J180" s="15" t="s">
+        <v>1153</v>
+      </c>
+      <c r="K180" s="15" t="s">
+        <v>1154</v>
+      </c>
+      <c r="L180" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="M180" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="N180" s="3" t="str">
+        <f t="shared" si="14"/>
+        <v>true</v>
+      </c>
+      <c r="O180" s="3" t="str">
+        <f t="shared" si="11"/>
         <v>{ "workOsisID": "D&amp;C", "bookName": "D&amp;C", "bookSubtitle": "of The Church of Jesus Christ of Latter-day Saints", "bookOsisID": "D&amp;C", "paratext": null, "groups": ["Doctrine and Covenants","LDS"], "aliases": ["D and C", "The Doctrine &amp; Covenants","Doctrine &amp; Covenants", "The Doctrine and Covenants"], "chapterLabel": "Section", "verseLabel": "Verse", "authors": ["Joseph Smith"], "dateEarliest": "1823-09-21", "dateLatest": "1841-01-19", "hasData": true, "traditions": ["lds"] },</v>
-      </c>
-    </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A179" t="s">
-        <v>634</v>
-      </c>
-      <c r="I179" s="7" t="s">
-        <v>1084</v>
-      </c>
-      <c r="J179" s="14" t="s">
-        <v>1078</v>
-      </c>
-      <c r="K179" s="14" t="s">
-        <v>1079</v>
-      </c>
-    </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A180" t="s">
-        <v>605</v>
-      </c>
-      <c r="I180" s="7" t="s">
-        <v>1084</v>
-      </c>
-      <c r="J180" s="14" t="s">
-        <v>1080</v>
-      </c>
-      <c r="K180" s="14" t="s">
-        <v>1081</v>
       </c>
     </row>
     <row r="181" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>606</v>
+        <v>634</v>
       </c>
       <c r="I181" s="7" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J181" s="14" t="s">
-        <v>1133</v>
+        <v>1078</v>
       </c>
       <c r="K181" s="14" t="s">
-        <v>1010</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="182" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="I182" s="7" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="J182" s="14" t="s">
-        <v>1133</v>
+        <v>1080</v>
       </c>
       <c r="K182" s="14" t="s">
-        <v>1134</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="183" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="I183" s="7" t="s">
         <v>1085</v>
       </c>
       <c r="J183" s="14" t="s">
-        <v>1008</v>
+        <v>1133</v>
       </c>
       <c r="K183" s="14" t="s">
-        <v>1022</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="184" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="I184" s="7" t="s">
         <v>1085</v>
       </c>
       <c r="J184" s="14" t="s">
-        <v>1029</v>
+        <v>1133</v>
       </c>
       <c r="K184" s="14" t="s">
-        <v>1073</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="185" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="I185" s="7" t="s">
         <v>1085</v>
       </c>
       <c r="J185" s="14" t="s">
-        <v>1013</v>
+        <v>1008</v>
       </c>
       <c r="K185" s="14" t="s">
-        <v>1082</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="186" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="I186" s="7" t="s">
         <v>1085</v>
       </c>
       <c r="J186" s="14" t="s">
-        <v>1013</v>
+        <v>1029</v>
       </c>
       <c r="K186" s="14" t="s">
-        <v>1083</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="187" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="I187" s="7" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="J187" s="14" t="s">
-        <v>1021</v>
+        <v>1013</v>
       </c>
       <c r="K187" s="14" t="s">
-        <v>1073</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="188" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="I188" s="7" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="J188" s="14" t="s">
-        <v>1021</v>
+        <v>1013</v>
       </c>
       <c r="K188" s="14" t="s">
-        <v>1022</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="189" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="I189" s="7" t="s">
         <v>1086</v>
@@ -12887,29 +12974,29 @@
         <v>1021</v>
       </c>
       <c r="K189" s="14" t="s">
-        <v>1019</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="190" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="I190" s="7" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="J190" s="14" t="s">
-        <v>1032</v>
+        <v>1021</v>
       </c>
       <c r="K190" s="14" t="s">
-        <v>1073</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="191" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="I191" s="7" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="J191" s="14" t="s">
         <v>1021</v>
@@ -12920,7 +13007,7 @@
     </row>
     <row r="192" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="I192" s="7" t="s">
         <v>1087</v>
@@ -12929,46 +13016,46 @@
         <v>1032</v>
       </c>
       <c r="K192" s="14" t="s">
-        <v>1019</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="193" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="I193" s="7" t="s">
         <v>1087</v>
       </c>
       <c r="J193" s="14" t="s">
-        <v>1014</v>
+        <v>1021</v>
       </c>
       <c r="K193" s="14" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="194" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="I194" s="7" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="J194" s="14" t="s">
-        <v>583</v>
+        <v>1032</v>
       </c>
       <c r="K194" s="14" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="195" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="I195" s="7" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="J195" s="14" t="s">
-        <v>1135</v>
+        <v>1014</v>
       </c>
       <c r="K195" s="14" t="s">
         <v>1017</v>
@@ -12976,188 +13063,216 @@
     </row>
     <row r="196" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="I196" s="7" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="J196" s="14" t="s">
-        <v>1136</v>
+        <v>583</v>
       </c>
       <c r="K196" s="14" t="s">
-        <v>1022</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="197" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="I197" s="7" t="s">
-        <v>1093</v>
+        <v>1088</v>
       </c>
       <c r="J197" s="14" t="s">
-        <v>1006</v>
+        <v>1135</v>
       </c>
       <c r="K197" s="14" t="s">
-        <v>1022</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="198" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="I198" s="7" t="s">
         <v>1089</v>
       </c>
       <c r="J198" s="14" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="K198" s="14" t="s">
-        <v>1138</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="199" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="I199" s="7" t="s">
-        <v>1090</v>
+        <v>1093</v>
       </c>
       <c r="J199" s="14" t="s">
-        <v>1032</v>
+        <v>1006</v>
       </c>
       <c r="K199" s="14" t="s">
-        <v>1139</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="200" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="I200" s="7" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="J200" s="14" t="s">
-        <v>1140</v>
+        <v>1137</v>
       </c>
       <c r="K200" s="14" t="s">
-        <v>1141</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="201" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="I201" s="7" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="J201" s="14" t="s">
-        <v>1142</v>
+        <v>1032</v>
       </c>
       <c r="K201" s="14" t="s">
-        <v>1143</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="202" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="I202" s="7" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="J202" s="14" t="s">
-        <v>1144</v>
+        <v>1140</v>
       </c>
       <c r="K202" s="14" t="s">
-        <v>1145</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="203" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="I203" s="7" t="s">
         <v>1091</v>
       </c>
       <c r="J203" s="14" t="s">
-        <v>1146</v>
+        <v>1142</v>
       </c>
       <c r="K203" s="14" t="s">
-        <v>1107</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="204" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="I204" s="7" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="J204" s="14" t="s">
-        <v>1140</v>
+        <v>1144</v>
       </c>
       <c r="K204" s="14" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="205" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="I205" s="7" t="s">
-        <v>1094</v>
+        <v>1091</v>
       </c>
       <c r="J205" s="14" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="K205" s="14" t="s">
-        <v>1149</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="206" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="I206" s="7" t="s">
         <v>1092</v>
       </c>
       <c r="J206" s="14" t="s">
-        <v>1150</v>
+        <v>1140</v>
       </c>
       <c r="K206" s="14" t="s">
-        <v>1151</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="207" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="I207" s="7" t="s">
-        <v>1092</v>
+        <v>1094</v>
       </c>
       <c r="J207" s="14" t="s">
         <v>1148</v>
       </c>
       <c r="K207" s="14" t="s">
-        <v>1145</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="208" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
+        <v>631</v>
+      </c>
+      <c r="I208" s="7" t="s">
+        <v>1092</v>
+      </c>
+      <c r="J208" s="14" t="s">
+        <v>1150</v>
+      </c>
+      <c r="K208" s="14" t="s">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="209" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A209" t="s">
+        <v>632</v>
+      </c>
+      <c r="I209" s="7" t="s">
+        <v>1092</v>
+      </c>
+      <c r="J209" s="14" t="s">
+        <v>1148</v>
+      </c>
+      <c r="K209" s="14" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="210" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A210" t="s">
         <v>633</v>
       </c>
-      <c r="I208" s="7" t="s">
+      <c r="I210" s="7" t="s">
         <v>1095</v>
       </c>
-      <c r="J208" s="14" t="s">
+      <c r="J210" s="14" t="s">
         <v>1152</v>
       </c>
-      <c r="K208" s="14" t="s">
+      <c r="K210" s="14" t="s">
         <v>1134</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E178" xr:uid="{2457BBF2-065A-6B4B-8450-DD145766C676}"/>
+  <autoFilter ref="A1:E180" xr:uid="{2457BBF2-065A-6B4B-8450-DD145766C676}"/>
   <hyperlinks>
     <hyperlink ref="A18" r:id="rId1" location="cite_note-6" display="https://wiki.crosswire.org/OSIS_Book_Abbreviations - cite_note-6" xr:uid="{413E20E8-A50F-EA4D-8B77-20FFD74AB053}"/>
   </hyperlinks>
@@ -13322,7 +13437,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{666CD579-589B-8442-BE20-716F9EAF0623}">
-  <dimension ref="B1:I9"/>
+  <dimension ref="B1:I11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
@@ -13399,7 +13514,7 @@
         <v>true</v>
       </c>
       <c r="I3" t="str">
-        <f t="shared" ref="I3:I9" si="1">"{ ""workOsisID"": """&amp;B3&amp;""", ""workTitle"": """&amp;C3&amp;""", ""workSubtitle"": """&amp;D3&amp;""", ""aliases"": "&amp;E3&amp;", ""hasData"": "&amp;H3&amp;" },"</f>
+        <f t="shared" ref="I3:I11" si="1">"{ ""workOsisID"": """&amp;B3&amp;""", ""workTitle"": """&amp;C3&amp;""", ""workSubtitle"": """&amp;D3&amp;""", ""aliases"": "&amp;E3&amp;", ""hasData"": "&amp;H3&amp;" },"</f>
         <v>{ "workOsisID": "KJVA", "workTitle": "The Holy Bible Apocrypha", "workSubtitle": "King James Version", "aliases": ["King James Apocrypha"], "hasData": true },</v>
       </c>
     </row>
@@ -13530,6 +13645,45 @@
       <c r="I9" t="str">
         <f t="shared" si="1"/>
         <v>{ "workOsisID": "Fathers", "workTitle": "Apostolic Fathers", "workSubtitle": "Translated by J.  B. Lightfoot", "aliases": ["The Apostolic Fathers"], "hasData": false },</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1293</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1294</v>
+      </c>
+      <c r="H10" s="19" t="s">
+        <v>1215</v>
+      </c>
+      <c r="I10" t="str">
+        <f t="shared" si="1"/>
+        <v>{ "workOsisID": "Jasher", "workTitle": "Jasher", "workSubtitle": "", "aliases": ["Sepir Ha Yasher","Sefer haYashar","The Book of Jasher","Book of Jasher"], "hasData": true },</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1297</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1302</v>
+      </c>
+      <c r="E11" t="s">
+        <v>1299</v>
+      </c>
+      <c r="H11" s="19" t="s">
+        <v>1215</v>
+      </c>
+      <c r="I11" t="str">
+        <f t="shared" si="1"/>
+        <v>{ "workOsisID": "AscIsa", "workTitle": "Ascension of Isaiah", "workSubtitle": "Translated by R. H. Charles", "aliases": ["The Ascension of Isaiah"], "hasData": true },</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
exclude book metadata from verse data files
</commit_message>
<xml_diff>
--- a/data/research/research.xlsx
+++ b/data/research/research.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ksnyder/Sites/public-domain-books/data/research/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B540EFB-3EAF-C94B-BBE0-DEC8ABB7AFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD84B17-0A10-574F-808B-CE58F04C01AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19420" xr2:uid="{948352A4-4516-F447-8F65-D2A52CDFF619}"/>
+    <workbookView xWindow="53100" yWindow="700" windowWidth="47220" windowHeight="25960" xr2:uid="{948352A4-4516-F447-8F65-D2A52CDFF619}"/>
   </bookViews>
   <sheets>
     <sheet name="Books" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3081" uniqueCount="1303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3081" uniqueCount="1304">
   <si>
     <t>Gen</t>
   </si>
@@ -3952,6 +3952,9 @@
   </si>
   <si>
     <t>["Song of the Three Children","Song of the Three Holy Children","Aza"]</t>
+  </si>
+  <si>
+    <t>["D and C","The Doctrine &amp; Covenants","Doctrine &amp; Covenants", "The Doctrine and Covenants"]</t>
   </si>
 </sst>
 </file>
@@ -12807,7 +12810,7 @@
     </row>
     <row r="180" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A180" s="3" t="s">
-        <v>451</v>
+        <v>568</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>567</v>
@@ -12819,7 +12822,7 @@
         <v>569</v>
       </c>
       <c r="F180" s="3" t="s">
-        <v>637</v>
+        <v>1303</v>
       </c>
       <c r="G180" s="6" t="s">
         <v>451</v>
@@ -12848,7 +12851,7 @@
       </c>
       <c r="O180" s="3" t="str">
         <f t="shared" si="11"/>
-        <v>{ "workOsisID": "D&amp;C", "bookName": "D&amp;C", "bookSubtitle": "of The Church of Jesus Christ of Latter-day Saints", "bookOsisID": "D&amp;C", "paratext": null, "groups": ["Doctrine and Covenants","LDS"], "aliases": ["D and C", "The Doctrine &amp; Covenants","Doctrine &amp; Covenants", "The Doctrine and Covenants"], "chapterLabel": "Section", "verseLabel": "Verse", "authors": ["Joseph Smith"], "dateEarliest": "1823-09-21", "dateLatest": "1841-01-19", "hasData": true, "traditions": ["lds"] },</v>
+        <v>{ "workOsisID": "D&amp;C", "bookName": "Doctrine and Covenants", "bookSubtitle": "of The Church of Jesus Christ of Latter-day Saints", "bookOsisID": "D&amp;C", "paratext": null, "groups": ["Doctrine and Covenants","LDS"], "aliases": ["D and C","The Doctrine &amp; Covenants","Doctrine &amp; Covenants", "The Doctrine and Covenants"], "chapterLabel": "Section", "verseLabel": "Verse", "authors": ["Joseph Smith"], "dateEarliest": "1823-09-21", "dateLatest": "1841-01-19", "hasData": true, "traditions": ["lds"] },</v>
       </c>
     </row>
     <row r="181" spans="1:15" x14ac:dyDescent="0.2">

</xml_diff>